<commit_message>
Mock 4: round 2 marks from the second review in Cowork (M4-S09 and M4-S43 good). The owner did not mark this round. The assistant typed the marks on the instruction of the owner.
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TnghEw2ou31QVRW6aTsXeq
</commit_message>
<xml_diff>
--- a/marking/M4-round2.xlsx
+++ b/marking/M4-round2.xlsx
@@ -596,7 +596,11 @@
 D: Stronger emphasis leaves the instruction just as general. The guide says general instructions fail because they lack specific categorical criteria, not because of their tone.</t>
         </is>
       </c>
-      <c r="N2" s="4" t="n"/>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O2" s="4" t="n"/>
     </row>
     <row r="3">
@@ -664,7 +668,11 @@
 D: More depth inside the same narrow subtasks still leaves refunds and pricing unassigned, so the coverage gap from the narrow decomposition remains.</t>
         </is>
       </c>
-      <c r="N3" s="4" t="n"/>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O3" s="4" t="n"/>
     </row>
   </sheetData>

</xml_diff>